<commit_message>
28: đồng bộ 07/10 — lọc nguồn câu hỏi luật, keo_drive, soffice, văn bản chỉ có bản chữ
</commit_message>
<xml_diff>
--- a/deploy/kiem-thu/KICH_BAN_KIEM_THU.xlsx
+++ b/deploy/kiem-thu/KICH_BAN_KIEM_THU.xlsx
@@ -10749,7 +10749,7 @@
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t>Điều 26 Luật Đầu tư 2020</t>
+          <t>Điều 26 Luật Đầu tư 2020 — THEO LUẬT HIỆN HÀNH (đề xuất, chờ luật sư HDS xác nhận): Điều 21 Luật Đầu tư 2025</t>
         </is>
       </c>
       <c r="G4" s="14" t="inlineStr"/>
@@ -10829,7 +10829,7 @@
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>Điều 46 Luật Đầu tư 2020; Luật Đất đai (đất thuê trả tiền hằng năm)</t>
+          <t>Điều 46 Luật Đầu tư 2020; Luật Đất đai (đất thuê trả tiền hằng năm) — THEO LUẬT HIỆN HÀNH (đề xuất, chờ luật sư HDS xác nhận): Điều 34 Luật Đầu tư 2025; Luật Đất đai (đất thuê trả tiền hằng năm)</t>
         </is>
       </c>
       <c r="G6" s="14" t="inlineStr"/>
@@ -10869,7 +10869,7 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Điều 202 LDN 2020</t>
+          <t>Điều 202 LDN 2020 — THEO LUẬT HIỆN HÀNH (đề xuất, chờ luật sư HDS xác nhận): Điều 204 LDN 2020</t>
         </is>
       </c>
       <c r="G7" s="14" t="inlineStr"/>
@@ -11917,7 +11917,7 @@
       </c>
       <c r="F33" s="14" t="inlineStr">
         <is>
-          <t>Điều 38, 39, 41 LDN 2020; Điều 19 NĐ 01/2021/NĐ-CP</t>
+          <t>Điều 38, 39, 41 LDN 2020; Điều 19 NĐ 01/2021/NĐ-CP — THEO LUẬT HIỆN HÀNH (đề xuất, chờ luật sư HDS xác nhận): Điều 38, 39, 41 LDN 2020; NĐ 168/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="G33" s="14" t="inlineStr">
@@ -12041,7 +12041,7 @@
       </c>
       <c r="F36" s="14" t="inlineStr">
         <is>
-          <t>Điều 57, 58 LDN 2020; NĐ 01/2021/NĐ-CP</t>
+          <t>Điều 57, 58 LDN 2020; NĐ 01/2021/NĐ-CP — THEO LUẬT HIỆN HÀNH (đề xuất, chờ luật sư HDS xác nhận): Điều 57, 58 LDN 2020; NĐ 168/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="G36" s="14" t="inlineStr"/>
@@ -12081,7 +12081,7 @@
       </c>
       <c r="F37" s="14" t="inlineStr">
         <is>
-          <t>Luật Quản lý thuế; Thông tư đăng ký thuế; Điều 47 NĐ 01/2021/NĐ-CP</t>
+          <t>Luật Quản lý thuế; Thông tư đăng ký thuế; Điều 47 NĐ 01/2021/NĐ-CP — THEO LUẬT HIỆN HÀNH (đề xuất, chờ luật sư HDS xác nhận): Luật Quản lý thuế 108/2025/QH15; NĐ 168/2025/NĐ-CP</t>
         </is>
       </c>
       <c r="G37" s="14" t="inlineStr"/>
@@ -12161,7 +12161,7 @@
       </c>
       <c r="F39" s="14" t="inlineStr">
         <is>
-          <t>Điều 22, 37, 38 Luật Đầu tư 2020; NĐ 31/2021/NĐ-CP</t>
+          <t>Điều 22, 37, 38 Luật Đầu tư 2020; NĐ 31/2021/NĐ-CP — THEO LUẬT HIỆN HÀNH (đề xuất, chờ luật sư HDS xác nhận): Điều 19, 26, 27 Luật Đầu tư 2025; NĐ 96/2026/NĐ-CP</t>
         </is>
       </c>
       <c r="G39" s="14" t="inlineStr">
@@ -12205,7 +12205,7 @@
       </c>
       <c r="F40" s="14" t="inlineStr">
         <is>
-          <t>Điều 29, 30, 31, 32 Luật Đầu tư 2020; Luật Đất đai</t>
+          <t>Điều 29, 30, 31, 32 Luật Đầu tư 2020; Luật Đất đai — THEO LUẬT HIỆN HÀNH (đề xuất, chờ luật sư HDS xác nhận): Điều 23, 24, 25 Luật Đầu tư 2025; Luật Đất đai</t>
         </is>
       </c>
       <c r="G40" s="14" t="inlineStr"/>
@@ -12245,7 +12245,7 @@
       </c>
       <c r="F41" s="14" t="inlineStr">
         <is>
-          <t>Điều 41, 44 Luật Đầu tư 2020</t>
+          <t>Điều 41, 44 Luật Đầu tư 2020 — THEO LUẬT HIỆN HÀNH (đề xuất, chờ luật sư HDS xác nhận): Điều 31, 33 Luật Đầu tư 2025</t>
         </is>
       </c>
       <c r="G41" s="14" t="inlineStr"/>
@@ -12285,7 +12285,7 @@
       </c>
       <c r="F42" s="14" t="inlineStr">
         <is>
-          <t>Điểm b khoản 2 Điều 26 Luật Đầu tư 2020; NĐ 31/2021/NĐ-CP</t>
+          <t>Điểm b khoản 2 Điều 26 Luật Đầu tư 2020; NĐ 31/2021/NĐ-CP — THEO LUẬT HIỆN HÀNH (đề xuất, chờ luật sư HDS xác nhận): Điều 21 Luật Đầu tư 2025; NĐ 96/2026/NĐ-CP</t>
         </is>
       </c>
       <c r="G42" s="14" t="inlineStr"/>

</xml_diff>